<commit_message>
funkcni check na ACQ
</commit_message>
<xml_diff>
--- a/data/input_fwdKrivka.xlsx
+++ b/data/input_fwdKrivka.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\krizova\Documents\R\02 cenoveKalkukacky\_vyvoj\shiny_app\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\krizova\Documents\R\02 cenoveKalkukacky\ZP\ZP_shiny_app\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4D1B358-680E-405D-AFFE-2E846CDB5E56}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87DF9926-85A4-4778-8B1D-4E8C6775C517}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="30720" windowHeight="13284" firstSheet="1" activeTab="1" xr2:uid="{F3DAE777-5404-4A54-B56B-E80B53D5C96F}"/>
   </bookViews>
@@ -133,7 +133,7 @@
     <numFmt numFmtId="164" formatCode="d/m/yyyy\ h:mm;@"/>
     <numFmt numFmtId="165" formatCode="0.0000"/>
     <numFmt numFmtId="166" formatCode="0.000"/>
-    <numFmt numFmtId="175" formatCode="0.0000000000000000"/>
+    <numFmt numFmtId="167" formatCode="0.0000000000000000"/>
   </numFmts>
   <fonts count="9" x14ac:knownFonts="1">
     <font>
@@ -291,7 +291,7 @@
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="175" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hypertextový odkaz" xfId="1" builtinId="8"/>
@@ -543,17 +543,18 @@
     <sheetNames>
       <sheetName val="Settings"/>
       <sheetName val="Forward"/>
+      <sheetName val="001_FWD_SPP-CZ_KAM_Aktual"/>
     </sheetNames>
     <definedNames>
       <definedName name="Refresh"/>
       <definedName name="Save"/>
     </definedNames>
     <sheetDataSet>
-      <sheetData sheetId="0" refreshError="1"/>
+      <sheetData sheetId="0"/>
       <sheetData sheetId="1">
         <row r="2">
           <cell r="C2">
-            <v>46037.434039351851</v>
+            <v>46050.386261574073</v>
           </cell>
         </row>
         <row r="6">
@@ -561,10 +562,10 @@
             <v>46023</v>
           </cell>
           <cell r="C6">
-            <v>32.728387096774206</v>
+            <v>35.913225806451614</v>
           </cell>
           <cell r="D6">
-            <v>24.245716399999999</v>
+            <v>24.227912250000003</v>
           </cell>
         </row>
         <row r="7">
@@ -572,10 +573,10 @@
             <v>46054</v>
           </cell>
           <cell r="C7">
-            <v>33.747999999999998</v>
+            <v>40.610999999999997</v>
           </cell>
           <cell r="D7">
-            <v>24.269803640000099</v>
+            <v>24.243947091004301</v>
           </cell>
         </row>
         <row r="8">
@@ -583,10 +584,10 @@
             <v>46082</v>
           </cell>
           <cell r="C8">
-            <v>33.106000000000002</v>
+            <v>39.448999999999998</v>
           </cell>
           <cell r="D8">
-            <v>24.293141819828548</v>
+            <v>24.266986128912897</v>
           </cell>
         </row>
         <row r="9">
@@ -594,10 +595,10 @@
             <v>46113</v>
           </cell>
           <cell r="C9">
-            <v>30.044</v>
+            <v>34.341999999999999</v>
           </cell>
           <cell r="D9">
-            <v>24.316521302545301</v>
+            <v>24.291457310664399</v>
           </cell>
         </row>
         <row r="10">
@@ -605,10 +606,10 @@
             <v>46143</v>
           </cell>
           <cell r="C10">
-            <v>28.521000000000001</v>
+            <v>31.01</v>
           </cell>
           <cell r="D10">
-            <v>24.3404291964079</v>
+            <v>24.315012617520551</v>
           </cell>
         </row>
         <row r="11">
@@ -616,10 +617,10 @@
             <v>46174</v>
           </cell>
           <cell r="C11">
-            <v>28.596</v>
+            <v>30.280999999999999</v>
           </cell>
           <cell r="D11">
-            <v>24.364349952196651</v>
+            <v>24.338008387952101</v>
           </cell>
         </row>
         <row r="12">
@@ -627,10 +628,10 @@
             <v>46204</v>
           </cell>
           <cell r="C12">
-            <v>28.225000000000001</v>
+            <v>30.103000000000002</v>
           </cell>
           <cell r="D12">
-            <v>24.386440854556451</v>
+            <v>24.359518182411151</v>
           </cell>
         </row>
         <row r="13">
@@ -638,10 +639,10 @@
             <v>46235</v>
           </cell>
           <cell r="C13">
-            <v>28.303999999999998</v>
+            <v>30.186</v>
           </cell>
           <cell r="D13">
-            <v>24.410428306904301</v>
+            <v>24.382257572546649</v>
           </cell>
         </row>
         <row r="14">
@@ -649,10 +650,10 @@
             <v>46266</v>
           </cell>
           <cell r="C14">
-            <v>28.574000000000002</v>
+            <v>30.375</v>
           </cell>
           <cell r="D14">
-            <v>24.430647486660551</v>
+            <v>24.401510875306251</v>
           </cell>
         </row>
         <row r="15">
@@ -660,10 +661,10 @@
             <v>46296</v>
           </cell>
           <cell r="C15">
-            <v>28.79</v>
+            <v>30.260999999999999</v>
           </cell>
           <cell r="D15">
-            <v>24.451396102134851</v>
+            <v>24.420580732202552</v>
           </cell>
         </row>
         <row r="16">
@@ -671,10 +672,10 @@
             <v>46327</v>
           </cell>
           <cell r="C16">
-            <v>29.135999999999999</v>
+            <v>31.035</v>
           </cell>
           <cell r="D16">
-            <v>24.474463276803249</v>
+            <v>24.4401272218557</v>
           </cell>
         </row>
         <row r="17">
@@ -682,10 +683,10 @@
             <v>46357</v>
           </cell>
           <cell r="C17">
-            <v>29.881</v>
+            <v>30.902000000000001</v>
           </cell>
           <cell r="D17">
-            <v>24.492735426739351</v>
+            <v>24.456528189491749</v>
           </cell>
         </row>
         <row r="18">
@@ -693,10 +694,10 @@
             <v>46388</v>
           </cell>
           <cell r="C18">
-            <v>29.673500882117079</v>
+            <v>31.299869330163219</v>
           </cell>
           <cell r="D18">
-            <v>24.509228811731752</v>
+            <v>24.475567727902899</v>
           </cell>
         </row>
         <row r="19">
@@ -704,10 +705,10 @@
             <v>46419</v>
           </cell>
           <cell r="C19">
-            <v>29.608937129109862</v>
+            <v>31.262293168176676</v>
           </cell>
           <cell r="D19">
-            <v>24.532420013715601</v>
+            <v>24.4950518757691</v>
           </cell>
         </row>
         <row r="20">
@@ -715,10 +716,10 @@
             <v>46447</v>
           </cell>
           <cell r="C20">
-            <v>28.905192221331191</v>
+            <v>30.440985627613639</v>
           </cell>
           <cell r="D20">
-            <v>24.552235979775652</v>
+            <v>24.512048237611651</v>
           </cell>
         </row>
         <row r="21">
@@ -726,10 +727,10 @@
             <v>46478</v>
           </cell>
           <cell r="C21">
-            <v>26.476519045709704</v>
+            <v>27.166491511643347</v>
           </cell>
           <cell r="D21">
-            <v>24.575000779378001</v>
+            <v>24.531569554210499</v>
           </cell>
         </row>
         <row r="22">
@@ -737,10 +738,10 @@
             <v>46508</v>
           </cell>
           <cell r="C22">
-            <v>25.570474378508422</v>
+            <v>26.033838628906082</v>
           </cell>
           <cell r="D22">
-            <v>24.598110933508249</v>
+            <v>24.5516213584323</v>
           </cell>
         </row>
         <row r="23">
@@ -748,10 +749,10 @@
             <v>46539</v>
           </cell>
           <cell r="C23">
-            <v>25.362794306335203</v>
+            <v>25.851325842114296</v>
           </cell>
           <cell r="D23">
-            <v>24.618983008701001</v>
+            <v>24.56969354493765</v>
           </cell>
         </row>
         <row r="24">
@@ -759,10 +760,10 @@
             <v>46569</v>
           </cell>
           <cell r="C24">
-            <v>25.347729430633521</v>
+            <v>25.908226887408208</v>
           </cell>
           <cell r="D24">
-            <v>24.640571411771401</v>
+            <v>24.588376437396651</v>
           </cell>
         </row>
         <row r="25">
@@ -770,10 +771,10 @@
             <v>46600</v>
           </cell>
           <cell r="C25">
-            <v>25.492997874899757</v>
+            <v>26.026323396508776</v>
           </cell>
           <cell r="D25">
-            <v>24.661109051744802</v>
+            <v>24.609908339797901</v>
           </cell>
         </row>
         <row r="26">
@@ -781,10 +782,10 @@
             <v>46631</v>
           </cell>
           <cell r="C26">
-            <v>25.753405012028868</v>
+            <v>26.176628044454954</v>
           </cell>
           <cell r="D26">
-            <v>24.679924180045653</v>
+            <v>24.631424491090499</v>
           </cell>
         </row>
         <row r="27">
@@ -792,10 +793,10 @@
             <v>46661</v>
           </cell>
           <cell r="C27">
-            <v>25.901901643945468</v>
+            <v>26.533064781013028</v>
           </cell>
           <cell r="D27">
-            <v>24.698731947681001</v>
+            <v>24.652934498840299</v>
           </cell>
         </row>
         <row r="28">
@@ -803,10 +804,10 @@
             <v>46692</v>
           </cell>
           <cell r="C28">
-            <v>26.687427305533276</v>
+            <v>27.128915349656801</v>
           </cell>
           <cell r="D28">
-            <v>24.722336889160349</v>
+            <v>24.67106496040045</v>
           </cell>
         </row>
         <row r="29">
@@ -814,10 +815,10 @@
             <v>46722</v>
           </cell>
           <cell r="C29">
-            <v>27.263120769847632</v>
+            <v>27.612037432340948</v>
           </cell>
           <cell r="D29">
-            <v>24.745958330253249</v>
+            <v>24.685334210569998</v>
           </cell>
         </row>
         <row r="30">
@@ -825,10 +826,10 @@
             <v>46753</v>
           </cell>
           <cell r="C30">
-            <v>27.814047145199236</v>
+            <v>28.064027084849055</v>
           </cell>
           <cell r="D30">
-            <v>24.772730621634899</v>
+            <v>24.701482464614351</v>
           </cell>
         </row>
         <row r="31">
@@ -836,10 +837,10 @@
             <v>46784</v>
           </cell>
           <cell r="C31">
-            <v>27.765187711169723</v>
+            <v>28.014329469900527</v>
           </cell>
           <cell r="D31">
-            <v>24.792830255214501</v>
+            <v>24.717027609701599</v>
           </cell>
         </row>
         <row r="32">
@@ -847,10 +848,10 @@
             <v>46813</v>
           </cell>
           <cell r="C32">
-            <v>27.016009722717232</v>
+            <v>27.262382948070574</v>
           </cell>
           <cell r="D32">
-            <v>24.813490454096851</v>
+            <v>24.735151483676599</v>
           </cell>
         </row>
         <row r="33">
@@ -858,10 +859,10 @@
             <v>46844</v>
           </cell>
           <cell r="C33">
-            <v>25.047517413928293</v>
+            <v>24.59815863365581</v>
           </cell>
           <cell r="D33">
-            <v>24.837710041818301</v>
+            <v>24.756390390477399</v>
           </cell>
         </row>
         <row r="34">
@@ -869,10 +870,10 @@
             <v>46874</v>
           </cell>
           <cell r="C34">
-            <v>24.222335861429901</v>
+            <v>23.623653227491126</v>
           </cell>
           <cell r="D34">
-            <v>24.856941156696902</v>
+            <v>24.773249066614</v>
           </cell>
         </row>
         <row r="35">
@@ -880,10 +881,10 @@
             <v>46905</v>
           </cell>
           <cell r="C35">
-            <v>24.064899907334812</v>
+            <v>23.484283829048504</v>
           </cell>
           <cell r="D35">
-            <v>24.879019047143849</v>
+            <v>24.792597120893653</v>
           </cell>
         </row>
         <row r="36">
@@ -891,10 +892,10 @@
             <v>46935</v>
           </cell>
           <cell r="C36">
-            <v>23.961752213272511</v>
+            <v>23.338432133003902</v>
           </cell>
           <cell r="D36">
-            <v>24.901806572860252</v>
+            <v>24.812560107808899</v>
           </cell>
         </row>
         <row r="37">
@@ -902,10 +903,10 @@
             <v>46966</v>
           </cell>
           <cell r="C37">
-            <v>24.157189949390549</v>
+            <v>23.532901061063374</v>
           </cell>
           <cell r="D37">
-            <v>24.922455526302649</v>
+            <v>24.830643493508649</v>
           </cell>
         </row>
         <row r="38">
@@ -913,10 +914,10 @@
             <v>46997</v>
           </cell>
           <cell r="C38">
-            <v>24.488348335590562</v>
+            <v>23.86241785583081</v>
           </cell>
           <cell r="D38">
-            <v>24.944526188443298</v>
+            <v>24.849965522870448</v>
           </cell>
         </row>
         <row r="39">
@@ -924,10 +925,10 @@
             <v>47027</v>
           </cell>
           <cell r="C39">
-            <v>24.663156532896146</v>
+            <v>24.025555678814033</v>
           </cell>
           <cell r="D39">
-            <v>24.966594414959097</v>
+            <v>24.869278782966401</v>
           </cell>
         </row>
         <row r="40">
@@ -935,10 +936,10 @@
             <v>47058</v>
           </cell>
           <cell r="C40">
-            <v>25.526339867417498</v>
+            <v>24.884460111076702</v>
           </cell>
           <cell r="D40">
-            <v>24.98794844416085</v>
+            <v>24.887960685163051</v>
           </cell>
         </row>
         <row r="41">
@@ -946,10 +947,10 @@
             <v>47088</v>
           </cell>
           <cell r="C41">
-            <v>25.917215339653577</v>
+            <v>25.273397967195642</v>
           </cell>
           <cell r="D41">
-            <v>25.009300192340248</v>
+            <v>24.906634374727851</v>
           </cell>
         </row>
         <row r="42">
@@ -957,10 +958,10 @@
             <v>47119</v>
           </cell>
           <cell r="C42">
-            <v>26.546114462368614</v>
+            <v>25.616164054954741</v>
           </cell>
           <cell r="D42">
-            <v>25.0320728762049</v>
+            <v>24.926543924784902</v>
           </cell>
         </row>
         <row r="43">
@@ -968,10 +969,10 @@
             <v>47150</v>
           </cell>
           <cell r="C43">
-            <v>26.689327097970885</v>
+            <v>25.756113452002396</v>
           </cell>
           <cell r="D43">
-            <v>25.053990216973801</v>
+            <v>24.945034379127549</v>
           </cell>
         </row>
         <row r="44">
@@ -979,10 +980,10 @@
             <v>47178</v>
           </cell>
           <cell r="C44">
-            <v>26.232148299702096</v>
+            <v>25.329755986578153</v>
           </cell>
           <cell r="D44">
-            <v>25.074578182154902</v>
+            <v>24.9621287284691</v>
           </cell>
         </row>
         <row r="45">
@@ -990,10 +991,10 @@
             <v>47209</v>
           </cell>
           <cell r="C45">
-            <v>24.330725153167329</v>
+            <v>23.48546160688041</v>
           </cell>
           <cell r="D45">
-            <v>25.098105863410151</v>
+            <v>24.981655059711898</v>
           </cell>
         </row>
         <row r="46">
@@ -1001,10 +1002,10 @@
             <v>47239</v>
           </cell>
           <cell r="C46">
-            <v>23.709402641785168</v>
+            <v>22.872504945392631</v>
           </cell>
           <cell r="D46">
-            <v>25.119426514558249</v>
+            <v>24.999341521202751</v>
           </cell>
         </row>
         <row r="47">
@@ -1012,10 +1013,10 @@
             <v>47270</v>
           </cell>
           <cell r="C47">
-            <v>23.092486673036927</v>
+            <v>22.270397074373665</v>
           </cell>
           <cell r="D47">
-            <v>25.14221617806335</v>
+            <v>25.018237985278951</v>
           </cell>
         </row>
         <row r="48">
@@ -1023,10 +1024,10 @@
             <v>47300</v>
           </cell>
           <cell r="C48">
-            <v>22.971306750604239</v>
+            <v>22.156484774451155</v>
           </cell>
           <cell r="D48">
-            <v>25.165004418278698</v>
+            <v>25.037124370863001</v>
           </cell>
         </row>
         <row r="49">
@@ -1034,10 +1035,10 @@
             <v>47331</v>
           </cell>
           <cell r="C49">
-            <v>23.197142060592434</v>
+            <v>22.422280140937008</v>
           </cell>
           <cell r="D49">
-            <v>25.187056198809351</v>
+            <v>25.055391922135549</v>
           </cell>
         </row>
         <row r="50">
@@ -1045,10 +1046,10 @@
             <v>47362</v>
           </cell>
           <cell r="C50">
-            <v>23.654320858861222</v>
+            <v>22.943022083439899</v>
           </cell>
           <cell r="D50">
-            <v>25.211311617840749</v>
+            <v>25.075475326774001</v>
           </cell>
         </row>
         <row r="51">
@@ -1056,10 +1057,10 @@
             <v>47392</v>
           </cell>
           <cell r="C51">
-            <v>24.115906199763923</v>
+            <v>23.340087814598355</v>
           </cell>
           <cell r="D51">
-            <v>25.23189070856505</v>
+            <v>25.092506834986651</v>
           </cell>
         </row>
         <row r="52">
@@ -1067,10 +1068,10 @@
             <v>47423</v>
           </cell>
           <cell r="C52">
-            <v>24.540035928278343</v>
+            <v>23.817434595226008</v>
           </cell>
           <cell r="D52">
-            <v>25.254673347446051</v>
+            <v>25.111353556827549</v>
           </cell>
         </row>
         <row r="53">
@@ -1078,13 +1079,14 @@
             <v>47453</v>
           </cell>
           <cell r="C53">
-            <v>24.909083873868809</v>
+            <v>24.186293471165552</v>
           </cell>
           <cell r="D53">
-            <v>25.278189417262599</v>
+            <v>25.1307976660325</v>
           </cell>
         </row>
       </sheetData>
+      <sheetData sheetId="2" refreshError="1"/>
     </sheetDataSet>
   </externalBook>
 </externalLink>
@@ -1436,7 +1438,7 @@
       </c>
       <c r="C3" s="5">
         <f ca="1">TODAY()</f>
-        <v>46038</v>
+        <v>46050</v>
       </c>
       <c r="E3" s="3">
         <f ca="1">YEAR(C3)</f>
@@ -1452,15 +1454,15 @@
       </c>
       <c r="H3" s="3" t="str">
         <f ca="1">RIGHT(C4,2)</f>
-        <v>16</v>
+        <v>28</v>
       </c>
       <c r="I3" s="3" t="str">
         <f ca="1">F3&amp;"_"&amp;H3&amp;"_"&amp;E3</f>
-        <v>01_16_2026</v>
+        <v>01_28_2026</v>
       </c>
       <c r="J3" s="3" t="str">
         <f ca="1">E3&amp;"_"&amp;F3&amp;"_"&amp;H3</f>
-        <v>2026_01_16</v>
+        <v>2026_01_28</v>
       </c>
       <c r="L3" s="3">
         <v>2</v>
@@ -1475,7 +1477,7 @@
       </c>
       <c r="C4" s="6" t="str">
         <f ca="1">_xlfn.CONCAT(RIGHT(YEAR(C3),2),TEXT(C3,"mm"),TEXT(C3,"dd"))</f>
-        <v>260116</v>
+        <v>260128</v>
       </c>
       <c r="D4" s="7"/>
       <c r="L4" s="3">
@@ -1514,7 +1516,7 @@
       </c>
       <c r="C7" s="9" t="str">
         <f ca="1">"\\Hqs0338\s_ba\OPR\SPO\Trading analyses\Kalkulacka data\"&amp;E3&amp;"\"&amp;G3&amp;"\"&amp;I3&amp;"\"</f>
-        <v>\\Hqs0338\s_ba\OPR\SPO\Trading analyses\Kalkulacka data\2026\01_Januar\01_16_2026\</v>
+        <v>\\Hqs0338\s_ba\OPR\SPO\Trading analyses\Kalkulacka data\2026\01_Januar\01_28_2026\</v>
       </c>
       <c r="L7" s="3">
         <v>6</v>
@@ -1693,817 +1695,817 @@
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" s="10">
         <f>'Propojeni na FWD v Pricingu'!A2</f>
-        <v>46037.434039351851</v>
+        <v>46050.386261574073</v>
       </c>
       <c r="B2" s="10">
         <v>46023</v>
       </c>
       <c r="C2">
         <f>'Propojeni na FWD v Pricingu'!C2</f>
-        <v>32.728387096774206</v>
+        <v>35.913225806451614</v>
       </c>
       <c r="D2" s="15">
         <f>'Propojeni na FWD v Pricingu'!D2</f>
-        <v>24.245716399999999</v>
+        <v>24.227912250000003</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" s="10">
         <f>'Propojeni na FWD v Pricingu'!A3</f>
-        <v>46037.434039351851</v>
+        <v>46050.386261574073</v>
       </c>
       <c r="B3" s="10">
         <v>46054</v>
       </c>
       <c r="C3">
         <f>'Propojeni na FWD v Pricingu'!C3</f>
-        <v>33.747999999999998</v>
+        <v>40.610999999999997</v>
       </c>
       <c r="D3" s="15">
         <f>'Propojeni na FWD v Pricingu'!D3</f>
-        <v>24.269803640000099</v>
+        <v>24.243947091004301</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" s="10">
         <f>'Propojeni na FWD v Pricingu'!A4</f>
-        <v>46037.434039351851</v>
+        <v>46050.386261574073</v>
       </c>
       <c r="B4" s="10">
         <v>46082</v>
       </c>
       <c r="C4">
         <f>'Propojeni na FWD v Pricingu'!C4</f>
-        <v>33.106000000000002</v>
+        <v>39.448999999999998</v>
       </c>
       <c r="D4" s="15">
         <f>'Propojeni na FWD v Pricingu'!D4</f>
-        <v>24.293141819828548</v>
+        <v>24.266986128912897</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" s="10">
         <f>'Propojeni na FWD v Pricingu'!A5</f>
-        <v>46037.434039351851</v>
+        <v>46050.386261574073</v>
       </c>
       <c r="B5" s="10">
         <v>46113</v>
       </c>
       <c r="C5">
         <f>'Propojeni na FWD v Pricingu'!C5</f>
-        <v>30.044</v>
+        <v>34.341999999999999</v>
       </c>
       <c r="D5" s="15">
         <f>'Propojeni na FWD v Pricingu'!D5</f>
-        <v>24.316521302545301</v>
+        <v>24.291457310664399</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" s="10">
         <f>'Propojeni na FWD v Pricingu'!A6</f>
-        <v>46037.434039351851</v>
+        <v>46050.386261574073</v>
       </c>
       <c r="B6" s="10">
         <v>46143</v>
       </c>
       <c r="C6">
         <f>'Propojeni na FWD v Pricingu'!C6</f>
-        <v>28.521000000000001</v>
+        <v>31.01</v>
       </c>
       <c r="D6" s="15">
         <f>'Propojeni na FWD v Pricingu'!D6</f>
-        <v>24.3404291964079</v>
+        <v>24.315012617520551</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" s="10">
         <f>'Propojeni na FWD v Pricingu'!A7</f>
-        <v>46037.434039351851</v>
+        <v>46050.386261574073</v>
       </c>
       <c r="B7" s="10">
         <v>46174</v>
       </c>
       <c r="C7">
         <f>'Propojeni na FWD v Pricingu'!C7</f>
-        <v>28.596</v>
+        <v>30.280999999999999</v>
       </c>
       <c r="D7" s="15">
         <f>'Propojeni na FWD v Pricingu'!D7</f>
-        <v>24.364349952196651</v>
+        <v>24.338008387952101</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" s="10">
         <f>'Propojeni na FWD v Pricingu'!A8</f>
-        <v>46037.434039351851</v>
+        <v>46050.386261574073</v>
       </c>
       <c r="B8" s="10">
         <v>46204</v>
       </c>
       <c r="C8">
         <f>'Propojeni na FWD v Pricingu'!C8</f>
-        <v>28.225000000000001</v>
+        <v>30.103000000000002</v>
       </c>
       <c r="D8" s="15">
         <f>'Propojeni na FWD v Pricingu'!D8</f>
-        <v>24.386440854556451</v>
+        <v>24.359518182411151</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" s="10">
         <f>'Propojeni na FWD v Pricingu'!A9</f>
-        <v>46037.434039351851</v>
+        <v>46050.386261574073</v>
       </c>
       <c r="B9" s="10">
         <v>46235</v>
       </c>
       <c r="C9">
         <f>'Propojeni na FWD v Pricingu'!C9</f>
-        <v>28.303999999999998</v>
+        <v>30.186</v>
       </c>
       <c r="D9" s="15">
         <f>'Propojeni na FWD v Pricingu'!D9</f>
-        <v>24.410428306904301</v>
+        <v>24.382257572546649</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A10" s="10">
         <f>'Propojeni na FWD v Pricingu'!A10</f>
-        <v>46037.434039351851</v>
+        <v>46050.386261574073</v>
       </c>
       <c r="B10" s="10">
         <v>46266</v>
       </c>
       <c r="C10">
         <f>'Propojeni na FWD v Pricingu'!C10</f>
-        <v>28.574000000000002</v>
+        <v>30.375</v>
       </c>
       <c r="D10" s="15">
         <f>'Propojeni na FWD v Pricingu'!D10</f>
-        <v>24.430647486660551</v>
+        <v>24.401510875306251</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11" s="10">
         <f>'Propojeni na FWD v Pricingu'!A11</f>
-        <v>46037.434039351851</v>
+        <v>46050.386261574073</v>
       </c>
       <c r="B11" s="10">
         <v>46296</v>
       </c>
       <c r="C11">
         <f>'Propojeni na FWD v Pricingu'!C11</f>
-        <v>28.79</v>
+        <v>30.260999999999999</v>
       </c>
       <c r="D11" s="15">
         <f>'Propojeni na FWD v Pricingu'!D11</f>
-        <v>24.451396102134851</v>
+        <v>24.420580732202552</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12" s="10">
         <f>'Propojeni na FWD v Pricingu'!A12</f>
-        <v>46037.434039351851</v>
+        <v>46050.386261574073</v>
       </c>
       <c r="B12" s="10">
         <v>46327</v>
       </c>
       <c r="C12">
         <f>'Propojeni na FWD v Pricingu'!C12</f>
-        <v>29.135999999999999</v>
+        <v>31.035</v>
       </c>
       <c r="D12" s="15">
         <f>'Propojeni na FWD v Pricingu'!D12</f>
-        <v>24.474463276803249</v>
+        <v>24.4401272218557</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A13" s="10">
         <f>'Propojeni na FWD v Pricingu'!A13</f>
-        <v>46037.434039351851</v>
+        <v>46050.386261574073</v>
       </c>
       <c r="B13" s="10">
         <v>46357</v>
       </c>
       <c r="C13">
         <f>'Propojeni na FWD v Pricingu'!C13</f>
-        <v>29.881</v>
+        <v>30.902000000000001</v>
       </c>
       <c r="D13" s="15">
         <f>'Propojeni na FWD v Pricingu'!D13</f>
-        <v>24.492735426739351</v>
+        <v>24.456528189491749</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A14" s="10">
         <f>'Propojeni na FWD v Pricingu'!A14</f>
-        <v>46037.434039351851</v>
+        <v>46050.386261574073</v>
       </c>
       <c r="B14" s="10">
         <v>46388</v>
       </c>
       <c r="C14">
         <f>'Propojeni na FWD v Pricingu'!C14</f>
-        <v>29.673500882117079</v>
+        <v>31.299869330163219</v>
       </c>
       <c r="D14" s="15">
         <f>'Propojeni na FWD v Pricingu'!D14</f>
-        <v>24.509228811731752</v>
+        <v>24.475567727902899</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A15" s="10">
         <f>'Propojeni na FWD v Pricingu'!A15</f>
-        <v>46037.434039351851</v>
+        <v>46050.386261574073</v>
       </c>
       <c r="B15" s="10">
         <v>46419</v>
       </c>
       <c r="C15">
         <f>'Propojeni na FWD v Pricingu'!C15</f>
-        <v>29.608937129109862</v>
+        <v>31.262293168176676</v>
       </c>
       <c r="D15" s="15">
         <f>'Propojeni na FWD v Pricingu'!D15</f>
-        <v>24.532420013715601</v>
+        <v>24.4950518757691</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A16" s="10">
         <f>'Propojeni na FWD v Pricingu'!A16</f>
-        <v>46037.434039351851</v>
+        <v>46050.386261574073</v>
       </c>
       <c r="B16" s="10">
         <v>46447</v>
       </c>
       <c r="C16">
         <f>'Propojeni na FWD v Pricingu'!C16</f>
-        <v>28.905192221331191</v>
+        <v>30.440985627613639</v>
       </c>
       <c r="D16" s="15">
         <f>'Propojeni na FWD v Pricingu'!D16</f>
-        <v>24.552235979775652</v>
+        <v>24.512048237611651</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A17" s="10">
         <f>'Propojeni na FWD v Pricingu'!A17</f>
-        <v>46037.434039351851</v>
+        <v>46050.386261574073</v>
       </c>
       <c r="B17" s="10">
         <v>46478</v>
       </c>
       <c r="C17">
         <f>'Propojeni na FWD v Pricingu'!C17</f>
-        <v>26.476519045709704</v>
+        <v>27.166491511643347</v>
       </c>
       <c r="D17" s="15">
         <f>'Propojeni na FWD v Pricingu'!D17</f>
-        <v>24.575000779378001</v>
+        <v>24.531569554210499</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A18" s="10">
         <f>'Propojeni na FWD v Pricingu'!A18</f>
-        <v>46037.434039351851</v>
+        <v>46050.386261574073</v>
       </c>
       <c r="B18" s="10">
         <v>46508</v>
       </c>
       <c r="C18">
         <f>'Propojeni na FWD v Pricingu'!C18</f>
-        <v>25.570474378508422</v>
+        <v>26.033838628906082</v>
       </c>
       <c r="D18" s="15">
         <f>'Propojeni na FWD v Pricingu'!D18</f>
-        <v>24.598110933508249</v>
+        <v>24.5516213584323</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A19" s="10">
         <f>'Propojeni na FWD v Pricingu'!A19</f>
-        <v>46037.434039351851</v>
+        <v>46050.386261574073</v>
       </c>
       <c r="B19" s="10">
         <v>46539</v>
       </c>
       <c r="C19">
         <f>'Propojeni na FWD v Pricingu'!C19</f>
-        <v>25.362794306335203</v>
+        <v>25.851325842114296</v>
       </c>
       <c r="D19" s="15">
         <f>'Propojeni na FWD v Pricingu'!D19</f>
-        <v>24.618983008701001</v>
+        <v>24.56969354493765</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A20" s="10">
         <f>'Propojeni na FWD v Pricingu'!A20</f>
-        <v>46037.434039351851</v>
+        <v>46050.386261574073</v>
       </c>
       <c r="B20" s="10">
         <v>46569</v>
       </c>
       <c r="C20">
         <f>'Propojeni na FWD v Pricingu'!C20</f>
-        <v>25.347729430633521</v>
+        <v>25.908226887408208</v>
       </c>
       <c r="D20" s="15">
         <f>'Propojeni na FWD v Pricingu'!D20</f>
-        <v>24.640571411771401</v>
+        <v>24.588376437396651</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A21" s="10">
         <f>'Propojeni na FWD v Pricingu'!A21</f>
-        <v>46037.434039351851</v>
+        <v>46050.386261574073</v>
       </c>
       <c r="B21" s="10">
         <v>46600</v>
       </c>
       <c r="C21">
         <f>'Propojeni na FWD v Pricingu'!C21</f>
-        <v>25.492997874899757</v>
+        <v>26.026323396508776</v>
       </c>
       <c r="D21" s="15">
         <f>'Propojeni na FWD v Pricingu'!D21</f>
-        <v>24.661109051744802</v>
+        <v>24.609908339797901</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A22" s="10">
         <f>'Propojeni na FWD v Pricingu'!A22</f>
-        <v>46037.434039351851</v>
+        <v>46050.386261574073</v>
       </c>
       <c r="B22" s="10">
         <v>46631</v>
       </c>
       <c r="C22">
         <f>'Propojeni na FWD v Pricingu'!C22</f>
-        <v>25.753405012028868</v>
+        <v>26.176628044454954</v>
       </c>
       <c r="D22" s="15">
         <f>'Propojeni na FWD v Pricingu'!D22</f>
-        <v>24.679924180045653</v>
+        <v>24.631424491090499</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A23" s="10">
         <f>'Propojeni na FWD v Pricingu'!A23</f>
-        <v>46037.434039351851</v>
+        <v>46050.386261574073</v>
       </c>
       <c r="B23" s="10">
         <v>46661</v>
       </c>
       <c r="C23">
         <f>'Propojeni na FWD v Pricingu'!C23</f>
-        <v>25.901901643945468</v>
+        <v>26.533064781013028</v>
       </c>
       <c r="D23" s="15">
         <f>'Propojeni na FWD v Pricingu'!D23</f>
-        <v>24.698731947681001</v>
+        <v>24.652934498840299</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A24" s="10">
         <f>'Propojeni na FWD v Pricingu'!A24</f>
-        <v>46037.434039351851</v>
+        <v>46050.386261574073</v>
       </c>
       <c r="B24" s="10">
         <v>46692</v>
       </c>
       <c r="C24">
         <f>'Propojeni na FWD v Pricingu'!C24</f>
-        <v>26.687427305533276</v>
+        <v>27.128915349656801</v>
       </c>
       <c r="D24" s="15">
         <f>'Propojeni na FWD v Pricingu'!D24</f>
-        <v>24.722336889160349</v>
+        <v>24.67106496040045</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A25" s="10">
         <f>'Propojeni na FWD v Pricingu'!A25</f>
-        <v>46037.434039351851</v>
+        <v>46050.386261574073</v>
       </c>
       <c r="B25" s="10">
         <v>46722</v>
       </c>
       <c r="C25">
         <f>'Propojeni na FWD v Pricingu'!C25</f>
-        <v>27.263120769847632</v>
+        <v>27.612037432340948</v>
       </c>
       <c r="D25" s="15">
         <f>'Propojeni na FWD v Pricingu'!D25</f>
-        <v>24.745958330253249</v>
+        <v>24.685334210569998</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A26" s="10">
         <f>'Propojeni na FWD v Pricingu'!A26</f>
-        <v>46037.434039351851</v>
+        <v>46050.386261574073</v>
       </c>
       <c r="B26" s="10">
         <v>46753</v>
       </c>
       <c r="C26">
         <f>'Propojeni na FWD v Pricingu'!C26</f>
-        <v>27.814047145199236</v>
+        <v>28.064027084849055</v>
       </c>
       <c r="D26" s="15">
         <f>'Propojeni na FWD v Pricingu'!D26</f>
-        <v>24.772730621634899</v>
+        <v>24.701482464614351</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A27" s="10">
         <f>'Propojeni na FWD v Pricingu'!A27</f>
-        <v>46037.434039351851</v>
+        <v>46050.386261574073</v>
       </c>
       <c r="B27" s="10">
         <v>46784</v>
       </c>
       <c r="C27">
         <f>'Propojeni na FWD v Pricingu'!C27</f>
-        <v>27.765187711169723</v>
+        <v>28.014329469900527</v>
       </c>
       <c r="D27" s="15">
         <f>'Propojeni na FWD v Pricingu'!D27</f>
-        <v>24.792830255214501</v>
+        <v>24.717027609701599</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A28" s="10">
         <f>'Propojeni na FWD v Pricingu'!A28</f>
-        <v>46037.434039351851</v>
+        <v>46050.386261574073</v>
       </c>
       <c r="B28" s="10">
         <v>46813</v>
       </c>
       <c r="C28">
         <f>'Propojeni na FWD v Pricingu'!C28</f>
-        <v>27.016009722717232</v>
+        <v>27.262382948070574</v>
       </c>
       <c r="D28" s="15">
         <f>'Propojeni na FWD v Pricingu'!D28</f>
-        <v>24.813490454096851</v>
+        <v>24.735151483676599</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A29" s="10">
         <f>'Propojeni na FWD v Pricingu'!A29</f>
-        <v>46037.434039351851</v>
+        <v>46050.386261574073</v>
       </c>
       <c r="B29" s="10">
         <v>46844</v>
       </c>
       <c r="C29">
         <f>'Propojeni na FWD v Pricingu'!C29</f>
-        <v>25.047517413928293</v>
+        <v>24.59815863365581</v>
       </c>
       <c r="D29" s="15">
         <f>'Propojeni na FWD v Pricingu'!D29</f>
-        <v>24.837710041818301</v>
+        <v>24.756390390477399</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A30" s="10">
         <f>'Propojeni na FWD v Pricingu'!A30</f>
-        <v>46037.434039351851</v>
+        <v>46050.386261574073</v>
       </c>
       <c r="B30" s="10">
         <v>46874</v>
       </c>
       <c r="C30">
         <f>'Propojeni na FWD v Pricingu'!C30</f>
-        <v>24.222335861429901</v>
+        <v>23.623653227491126</v>
       </c>
       <c r="D30" s="15">
         <f>'Propojeni na FWD v Pricingu'!D30</f>
-        <v>24.856941156696902</v>
+        <v>24.773249066614</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A31" s="10">
         <f>'Propojeni na FWD v Pricingu'!A31</f>
-        <v>46037.434039351851</v>
+        <v>46050.386261574073</v>
       </c>
       <c r="B31" s="10">
         <v>46905</v>
       </c>
       <c r="C31">
         <f>'Propojeni na FWD v Pricingu'!C31</f>
-        <v>24.064899907334812</v>
+        <v>23.484283829048504</v>
       </c>
       <c r="D31" s="15">
         <f>'Propojeni na FWD v Pricingu'!D31</f>
-        <v>24.879019047143849</v>
+        <v>24.792597120893653</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A32" s="10">
         <f>'Propojeni na FWD v Pricingu'!A32</f>
-        <v>46037.434039351851</v>
+        <v>46050.386261574073</v>
       </c>
       <c r="B32" s="10">
         <v>46935</v>
       </c>
       <c r="C32">
         <f>'Propojeni na FWD v Pricingu'!C32</f>
-        <v>23.961752213272511</v>
+        <v>23.338432133003902</v>
       </c>
       <c r="D32" s="15">
         <f>'Propojeni na FWD v Pricingu'!D32</f>
-        <v>24.901806572860252</v>
+        <v>24.812560107808899</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A33" s="10">
         <f>'Propojeni na FWD v Pricingu'!A33</f>
-        <v>46037.434039351851</v>
+        <v>46050.386261574073</v>
       </c>
       <c r="B33" s="10">
         <v>46966</v>
       </c>
       <c r="C33">
         <f>'Propojeni na FWD v Pricingu'!C33</f>
-        <v>24.157189949390549</v>
+        <v>23.532901061063374</v>
       </c>
       <c r="D33" s="15">
         <f>'Propojeni na FWD v Pricingu'!D33</f>
-        <v>24.922455526302649</v>
+        <v>24.830643493508649</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A34" s="10">
         <f>'Propojeni na FWD v Pricingu'!A34</f>
-        <v>46037.434039351851</v>
+        <v>46050.386261574073</v>
       </c>
       <c r="B34" s="10">
         <v>46997</v>
       </c>
       <c r="C34">
         <f>'Propojeni na FWD v Pricingu'!C34</f>
-        <v>24.488348335590562</v>
+        <v>23.86241785583081</v>
       </c>
       <c r="D34" s="15">
         <f>'Propojeni na FWD v Pricingu'!D34</f>
-        <v>24.944526188443298</v>
+        <v>24.849965522870448</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A35" s="10">
         <f>'Propojeni na FWD v Pricingu'!A35</f>
-        <v>46037.434039351851</v>
+        <v>46050.386261574073</v>
       </c>
       <c r="B35" s="10">
         <v>47027</v>
       </c>
       <c r="C35">
         <f>'Propojeni na FWD v Pricingu'!C35</f>
-        <v>24.663156532896146</v>
+        <v>24.025555678814033</v>
       </c>
       <c r="D35" s="15">
         <f>'Propojeni na FWD v Pricingu'!D35</f>
-        <v>24.966594414959097</v>
+        <v>24.869278782966401</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A36" s="10">
         <f>'Propojeni na FWD v Pricingu'!A36</f>
-        <v>46037.434039351851</v>
+        <v>46050.386261574073</v>
       </c>
       <c r="B36" s="10">
         <v>47058</v>
       </c>
       <c r="C36">
         <f>'Propojeni na FWD v Pricingu'!C36</f>
-        <v>25.526339867417498</v>
+        <v>24.884460111076702</v>
       </c>
       <c r="D36" s="15">
         <f>'Propojeni na FWD v Pricingu'!D36</f>
-        <v>24.98794844416085</v>
+        <v>24.887960685163051</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A37" s="10">
         <f>'Propojeni na FWD v Pricingu'!A37</f>
-        <v>46037.434039351851</v>
+        <v>46050.386261574073</v>
       </c>
       <c r="B37" s="10">
         <v>47088</v>
       </c>
       <c r="C37">
         <f>'Propojeni na FWD v Pricingu'!C37</f>
-        <v>25.917215339653577</v>
+        <v>25.273397967195642</v>
       </c>
       <c r="D37" s="15">
         <f>'Propojeni na FWD v Pricingu'!D37</f>
-        <v>25.009300192340248</v>
+        <v>24.906634374727851</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A38" s="10">
         <f>'Propojeni na FWD v Pricingu'!A38</f>
-        <v>46037.434039351851</v>
+        <v>46050.386261574073</v>
       </c>
       <c r="B38" s="10">
         <v>47119</v>
       </c>
       <c r="C38">
         <f>'Propojeni na FWD v Pricingu'!C38</f>
-        <v>26.546114462368614</v>
+        <v>25.616164054954741</v>
       </c>
       <c r="D38" s="15">
         <f>'Propojeni na FWD v Pricingu'!D38</f>
-        <v>25.0320728762049</v>
+        <v>24.926543924784902</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A39" s="10">
         <f>'Propojeni na FWD v Pricingu'!A39</f>
-        <v>46037.434039351851</v>
+        <v>46050.386261574073</v>
       </c>
       <c r="B39" s="10">
         <v>47150</v>
       </c>
       <c r="C39">
         <f>'Propojeni na FWD v Pricingu'!C39</f>
-        <v>26.689327097970885</v>
+        <v>25.756113452002396</v>
       </c>
       <c r="D39" s="15">
         <f>'Propojeni na FWD v Pricingu'!D39</f>
-        <v>25.053990216973801</v>
+        <v>24.945034379127549</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A40" s="10">
         <f>'Propojeni na FWD v Pricingu'!A40</f>
-        <v>46037.434039351851</v>
+        <v>46050.386261574073</v>
       </c>
       <c r="B40" s="10">
         <v>47178</v>
       </c>
       <c r="C40">
         <f>'Propojeni na FWD v Pricingu'!C40</f>
-        <v>26.232148299702096</v>
+        <v>25.329755986578153</v>
       </c>
       <c r="D40" s="15">
         <f>'Propojeni na FWD v Pricingu'!D40</f>
-        <v>25.074578182154902</v>
+        <v>24.9621287284691</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A41" s="10">
         <f>'Propojeni na FWD v Pricingu'!A41</f>
-        <v>46037.434039351851</v>
+        <v>46050.386261574073</v>
       </c>
       <c r="B41" s="10">
         <v>47209</v>
       </c>
       <c r="C41">
         <f>'Propojeni na FWD v Pricingu'!C41</f>
-        <v>24.330725153167329</v>
+        <v>23.48546160688041</v>
       </c>
       <c r="D41" s="15">
         <f>'Propojeni na FWD v Pricingu'!D41</f>
-        <v>25.098105863410151</v>
+        <v>24.981655059711898</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A42" s="10">
         <f>'Propojeni na FWD v Pricingu'!A42</f>
-        <v>46037.434039351851</v>
+        <v>46050.386261574073</v>
       </c>
       <c r="B42" s="10">
         <v>47239</v>
       </c>
       <c r="C42">
         <f>'Propojeni na FWD v Pricingu'!C42</f>
-        <v>23.709402641785168</v>
+        <v>22.872504945392631</v>
       </c>
       <c r="D42" s="15">
         <f>'Propojeni na FWD v Pricingu'!D42</f>
-        <v>25.119426514558249</v>
+        <v>24.999341521202751</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A43" s="10">
         <f>'Propojeni na FWD v Pricingu'!A43</f>
-        <v>46037.434039351851</v>
+        <v>46050.386261574073</v>
       </c>
       <c r="B43" s="10">
         <v>47270</v>
       </c>
       <c r="C43">
         <f>'Propojeni na FWD v Pricingu'!C43</f>
-        <v>23.092486673036927</v>
+        <v>22.270397074373665</v>
       </c>
       <c r="D43" s="15">
         <f>'Propojeni na FWD v Pricingu'!D43</f>
-        <v>25.14221617806335</v>
+        <v>25.018237985278951</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A44" s="10">
         <f>'Propojeni na FWD v Pricingu'!A44</f>
-        <v>46037.434039351851</v>
+        <v>46050.386261574073</v>
       </c>
       <c r="B44" s="10">
         <v>47300</v>
       </c>
       <c r="C44">
         <f>'Propojeni na FWD v Pricingu'!C44</f>
-        <v>22.971306750604239</v>
+        <v>22.156484774451155</v>
       </c>
       <c r="D44" s="15">
         <f>'Propojeni na FWD v Pricingu'!D44</f>
-        <v>25.165004418278698</v>
+        <v>25.037124370863001</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A45" s="10">
         <f>'Propojeni na FWD v Pricingu'!A45</f>
-        <v>46037.434039351851</v>
+        <v>46050.386261574073</v>
       </c>
       <c r="B45" s="10">
         <v>47331</v>
       </c>
       <c r="C45">
         <f>'Propojeni na FWD v Pricingu'!C45</f>
-        <v>23.197142060592434</v>
+        <v>22.422280140937008</v>
       </c>
       <c r="D45" s="15">
         <f>'Propojeni na FWD v Pricingu'!D45</f>
-        <v>25.187056198809351</v>
+        <v>25.055391922135549</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A46" s="10">
         <f>'Propojeni na FWD v Pricingu'!A46</f>
-        <v>46037.434039351851</v>
+        <v>46050.386261574073</v>
       </c>
       <c r="B46" s="10">
         <v>47362</v>
       </c>
       <c r="C46">
         <f>'Propojeni na FWD v Pricingu'!C46</f>
-        <v>23.654320858861222</v>
+        <v>22.943022083439899</v>
       </c>
       <c r="D46" s="15">
         <f>'Propojeni na FWD v Pricingu'!D46</f>
-        <v>25.211311617840749</v>
+        <v>25.075475326774001</v>
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A47" s="10">
         <f>'Propojeni na FWD v Pricingu'!A47</f>
-        <v>46037.434039351851</v>
+        <v>46050.386261574073</v>
       </c>
       <c r="B47" s="10">
         <v>47392</v>
       </c>
       <c r="C47">
         <f>'Propojeni na FWD v Pricingu'!C47</f>
-        <v>24.115906199763923</v>
+        <v>23.340087814598355</v>
       </c>
       <c r="D47" s="15">
         <f>'Propojeni na FWD v Pricingu'!D47</f>
-        <v>25.23189070856505</v>
+        <v>25.092506834986651</v>
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A48" s="10">
         <f>'Propojeni na FWD v Pricingu'!A48</f>
-        <v>46037.434039351851</v>
+        <v>46050.386261574073</v>
       </c>
       <c r="B48" s="10">
         <v>47423</v>
       </c>
       <c r="C48">
         <f>'Propojeni na FWD v Pricingu'!C48</f>
-        <v>24.540035928278343</v>
+        <v>23.817434595226008</v>
       </c>
       <c r="D48" s="15">
         <f>'Propojeni na FWD v Pricingu'!D48</f>
-        <v>25.254673347446051</v>
+        <v>25.111353556827549</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A49" s="10">
         <f>'Propojeni na FWD v Pricingu'!A49</f>
-        <v>46037.434039351851</v>
+        <v>46050.386261574073</v>
       </c>
       <c r="B49" s="10">
         <v>47453</v>
       </c>
       <c r="C49">
         <f>'Propojeni na FWD v Pricingu'!C49</f>
-        <v>24.909083873868809</v>
+        <v>24.186293471165552</v>
       </c>
       <c r="D49" s="15">
         <f>'Propojeni na FWD v Pricingu'!D49</f>
-        <v>25.278189417262599</v>
+        <v>25.1307976660325</v>
       </c>
     </row>
   </sheetData>
@@ -2538,7 +2540,7 @@
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" s="12">
         <f>[1]Forward!$C$2</f>
-        <v>46037.434039351851</v>
+        <v>46050.386261574073</v>
       </c>
       <c r="B2" s="12">
         <f>[1]Forward!$B$6</f>
@@ -2546,17 +2548,17 @@
       </c>
       <c r="C2" s="13">
         <f>[1]Forward!C6</f>
-        <v>32.728387096774206</v>
+        <v>35.913225806451614</v>
       </c>
       <c r="D2" s="14">
         <f>[1]Forward!D6</f>
-        <v>24.245716399999999</v>
+        <v>24.227912250000003</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" s="12">
         <f>[1]Forward!$C$2</f>
-        <v>46037.434039351851</v>
+        <v>46050.386261574073</v>
       </c>
       <c r="B3" s="12">
         <f>[1]Forward!$B$7</f>
@@ -2564,17 +2566,17 @@
       </c>
       <c r="C3" s="13">
         <f>[1]Forward!C7</f>
-        <v>33.747999999999998</v>
+        <v>40.610999999999997</v>
       </c>
       <c r="D3" s="14">
         <f>[1]Forward!D7</f>
-        <v>24.269803640000099</v>
+        <v>24.243947091004301</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" s="12">
         <f>[1]Forward!$C$2</f>
-        <v>46037.434039351851</v>
+        <v>46050.386261574073</v>
       </c>
       <c r="B4" s="12">
         <f>[1]Forward!$B$8</f>
@@ -2582,17 +2584,17 @@
       </c>
       <c r="C4" s="13">
         <f>[1]Forward!C8</f>
-        <v>33.106000000000002</v>
+        <v>39.448999999999998</v>
       </c>
       <c r="D4" s="14">
         <f>[1]Forward!D8</f>
-        <v>24.293141819828548</v>
+        <v>24.266986128912897</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" s="12">
         <f>[1]Forward!$C$2</f>
-        <v>46037.434039351851</v>
+        <v>46050.386261574073</v>
       </c>
       <c r="B5" s="12">
         <f>[1]Forward!$B$9</f>
@@ -2600,17 +2602,17 @@
       </c>
       <c r="C5" s="13">
         <f>[1]Forward!C9</f>
-        <v>30.044</v>
+        <v>34.341999999999999</v>
       </c>
       <c r="D5" s="14">
         <f>[1]Forward!D9</f>
-        <v>24.316521302545301</v>
+        <v>24.291457310664399</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" s="12">
         <f>[1]Forward!$C$2</f>
-        <v>46037.434039351851</v>
+        <v>46050.386261574073</v>
       </c>
       <c r="B6" s="12">
         <f>[1]Forward!$B$10</f>
@@ -2618,17 +2620,17 @@
       </c>
       <c r="C6" s="13">
         <f>[1]Forward!C10</f>
-        <v>28.521000000000001</v>
+        <v>31.01</v>
       </c>
       <c r="D6" s="14">
         <f>[1]Forward!D10</f>
-        <v>24.3404291964079</v>
+        <v>24.315012617520551</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" s="12">
         <f>[1]Forward!$C$2</f>
-        <v>46037.434039351851</v>
+        <v>46050.386261574073</v>
       </c>
       <c r="B7" s="12">
         <f>[1]Forward!$B$11</f>
@@ -2636,17 +2638,17 @@
       </c>
       <c r="C7" s="13">
         <f>[1]Forward!C11</f>
-        <v>28.596</v>
+        <v>30.280999999999999</v>
       </c>
       <c r="D7" s="14">
         <f>[1]Forward!D11</f>
-        <v>24.364349952196651</v>
+        <v>24.338008387952101</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" s="12">
         <f>[1]Forward!$C$2</f>
-        <v>46037.434039351851</v>
+        <v>46050.386261574073</v>
       </c>
       <c r="B8" s="12">
         <f>[1]Forward!$B$12</f>
@@ -2654,17 +2656,17 @@
       </c>
       <c r="C8" s="13">
         <f>[1]Forward!C12</f>
-        <v>28.225000000000001</v>
+        <v>30.103000000000002</v>
       </c>
       <c r="D8" s="14">
         <f>[1]Forward!D12</f>
-        <v>24.386440854556451</v>
+        <v>24.359518182411151</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" s="12">
         <f>[1]Forward!$C$2</f>
-        <v>46037.434039351851</v>
+        <v>46050.386261574073</v>
       </c>
       <c r="B9" s="12">
         <f>[1]Forward!B13</f>
@@ -2672,17 +2674,17 @@
       </c>
       <c r="C9" s="13">
         <f>[1]Forward!C13</f>
-        <v>28.303999999999998</v>
+        <v>30.186</v>
       </c>
       <c r="D9" s="14">
         <f>[1]Forward!D13</f>
-        <v>24.410428306904301</v>
+        <v>24.382257572546649</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A10" s="12">
         <f>[1]Forward!$C$2</f>
-        <v>46037.434039351851</v>
+        <v>46050.386261574073</v>
       </c>
       <c r="B10" s="12">
         <f>[1]Forward!B14</f>
@@ -2690,17 +2692,17 @@
       </c>
       <c r="C10" s="13">
         <f>[1]Forward!C14</f>
-        <v>28.574000000000002</v>
+        <v>30.375</v>
       </c>
       <c r="D10" s="14">
         <f>[1]Forward!D14</f>
-        <v>24.430647486660551</v>
+        <v>24.401510875306251</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11" s="12">
         <f>[1]Forward!$C$2</f>
-        <v>46037.434039351851</v>
+        <v>46050.386261574073</v>
       </c>
       <c r="B11" s="12">
         <f>[1]Forward!B15</f>
@@ -2708,17 +2710,17 @@
       </c>
       <c r="C11" s="13">
         <f>[1]Forward!C15</f>
-        <v>28.79</v>
+        <v>30.260999999999999</v>
       </c>
       <c r="D11" s="14">
         <f>[1]Forward!D15</f>
-        <v>24.451396102134851</v>
+        <v>24.420580732202552</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12" s="12">
         <f>[1]Forward!$C$2</f>
-        <v>46037.434039351851</v>
+        <v>46050.386261574073</v>
       </c>
       <c r="B12" s="12">
         <f>[1]Forward!B16</f>
@@ -2726,17 +2728,17 @@
       </c>
       <c r="C12" s="13">
         <f>[1]Forward!C16</f>
-        <v>29.135999999999999</v>
+        <v>31.035</v>
       </c>
       <c r="D12" s="14">
         <f>[1]Forward!D16</f>
-        <v>24.474463276803249</v>
+        <v>24.4401272218557</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A13" s="12">
         <f>[1]Forward!$C$2</f>
-        <v>46037.434039351851</v>
+        <v>46050.386261574073</v>
       </c>
       <c r="B13" s="12">
         <f>[1]Forward!B17</f>
@@ -2744,17 +2746,17 @@
       </c>
       <c r="C13" s="13">
         <f>[1]Forward!C17</f>
-        <v>29.881</v>
+        <v>30.902000000000001</v>
       </c>
       <c r="D13" s="14">
         <f>[1]Forward!D17</f>
-        <v>24.492735426739351</v>
+        <v>24.456528189491749</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A14" s="12">
         <f>[1]Forward!$C$2</f>
-        <v>46037.434039351851</v>
+        <v>46050.386261574073</v>
       </c>
       <c r="B14" s="12">
         <f>[1]Forward!B18</f>
@@ -2762,17 +2764,17 @@
       </c>
       <c r="C14" s="13">
         <f>[1]Forward!C18</f>
-        <v>29.673500882117079</v>
+        <v>31.299869330163219</v>
       </c>
       <c r="D14" s="14">
         <f>[1]Forward!D18</f>
-        <v>24.509228811731752</v>
+        <v>24.475567727902899</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A15" s="12">
         <f>[1]Forward!$C$2</f>
-        <v>46037.434039351851</v>
+        <v>46050.386261574073</v>
       </c>
       <c r="B15" s="12">
         <f>[1]Forward!B19</f>
@@ -2780,17 +2782,17 @@
       </c>
       <c r="C15" s="13">
         <f>[1]Forward!C19</f>
-        <v>29.608937129109862</v>
+        <v>31.262293168176676</v>
       </c>
       <c r="D15" s="14">
         <f>[1]Forward!D19</f>
-        <v>24.532420013715601</v>
+        <v>24.4950518757691</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A16" s="12">
         <f>[1]Forward!$C$2</f>
-        <v>46037.434039351851</v>
+        <v>46050.386261574073</v>
       </c>
       <c r="B16" s="12">
         <f>[1]Forward!B20</f>
@@ -2798,17 +2800,17 @@
       </c>
       <c r="C16" s="13">
         <f>[1]Forward!C20</f>
-        <v>28.905192221331191</v>
+        <v>30.440985627613639</v>
       </c>
       <c r="D16" s="14">
         <f>[1]Forward!D20</f>
-        <v>24.552235979775652</v>
+        <v>24.512048237611651</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A17" s="12">
         <f>[1]Forward!$C$2</f>
-        <v>46037.434039351851</v>
+        <v>46050.386261574073</v>
       </c>
       <c r="B17" s="12">
         <f>[1]Forward!B21</f>
@@ -2816,17 +2818,17 @@
       </c>
       <c r="C17" s="13">
         <f>[1]Forward!C21</f>
-        <v>26.476519045709704</v>
+        <v>27.166491511643347</v>
       </c>
       <c r="D17" s="14">
         <f>[1]Forward!D21</f>
-        <v>24.575000779378001</v>
+        <v>24.531569554210499</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A18" s="12">
         <f>[1]Forward!$C$2</f>
-        <v>46037.434039351851</v>
+        <v>46050.386261574073</v>
       </c>
       <c r="B18" s="12">
         <f>[1]Forward!B22</f>
@@ -2834,17 +2836,17 @@
       </c>
       <c r="C18" s="13">
         <f>[1]Forward!C22</f>
-        <v>25.570474378508422</v>
+        <v>26.033838628906082</v>
       </c>
       <c r="D18" s="14">
         <f>[1]Forward!D22</f>
-        <v>24.598110933508249</v>
+        <v>24.5516213584323</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A19" s="12">
         <f>[1]Forward!$C$2</f>
-        <v>46037.434039351851</v>
+        <v>46050.386261574073</v>
       </c>
       <c r="B19" s="12">
         <f>[1]Forward!B23</f>
@@ -2852,17 +2854,17 @@
       </c>
       <c r="C19" s="13">
         <f>[1]Forward!C23</f>
-        <v>25.362794306335203</v>
+        <v>25.851325842114296</v>
       </c>
       <c r="D19" s="14">
         <f>[1]Forward!D23</f>
-        <v>24.618983008701001</v>
+        <v>24.56969354493765</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A20" s="12">
         <f>[1]Forward!$C$2</f>
-        <v>46037.434039351851</v>
+        <v>46050.386261574073</v>
       </c>
       <c r="B20" s="12">
         <f>[1]Forward!B24</f>
@@ -2870,17 +2872,17 @@
       </c>
       <c r="C20" s="13">
         <f>[1]Forward!C24</f>
-        <v>25.347729430633521</v>
+        <v>25.908226887408208</v>
       </c>
       <c r="D20" s="14">
         <f>[1]Forward!D24</f>
-        <v>24.640571411771401</v>
+        <v>24.588376437396651</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A21" s="12">
         <f>[1]Forward!$C$2</f>
-        <v>46037.434039351851</v>
+        <v>46050.386261574073</v>
       </c>
       <c r="B21" s="12">
         <f>[1]Forward!B25</f>
@@ -2888,17 +2890,17 @@
       </c>
       <c r="C21" s="13">
         <f>[1]Forward!C25</f>
-        <v>25.492997874899757</v>
+        <v>26.026323396508776</v>
       </c>
       <c r="D21" s="14">
         <f>[1]Forward!D25</f>
-        <v>24.661109051744802</v>
+        <v>24.609908339797901</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A22" s="12">
         <f>[1]Forward!$C$2</f>
-        <v>46037.434039351851</v>
+        <v>46050.386261574073</v>
       </c>
       <c r="B22" s="12">
         <f>[1]Forward!B26</f>
@@ -2906,17 +2908,17 @@
       </c>
       <c r="C22" s="13">
         <f>[1]Forward!C26</f>
-        <v>25.753405012028868</v>
+        <v>26.176628044454954</v>
       </c>
       <c r="D22" s="14">
         <f>[1]Forward!D26</f>
-        <v>24.679924180045653</v>
+        <v>24.631424491090499</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A23" s="12">
         <f>[1]Forward!$C$2</f>
-        <v>46037.434039351851</v>
+        <v>46050.386261574073</v>
       </c>
       <c r="B23" s="12">
         <f>[1]Forward!B27</f>
@@ -2924,17 +2926,17 @@
       </c>
       <c r="C23" s="13">
         <f>[1]Forward!C27</f>
-        <v>25.901901643945468</v>
+        <v>26.533064781013028</v>
       </c>
       <c r="D23" s="14">
         <f>[1]Forward!D27</f>
-        <v>24.698731947681001</v>
+        <v>24.652934498840299</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A24" s="12">
         <f>[1]Forward!$C$2</f>
-        <v>46037.434039351851</v>
+        <v>46050.386261574073</v>
       </c>
       <c r="B24" s="12">
         <f>[1]Forward!B28</f>
@@ -2942,17 +2944,17 @@
       </c>
       <c r="C24" s="13">
         <f>[1]Forward!C28</f>
-        <v>26.687427305533276</v>
+        <v>27.128915349656801</v>
       </c>
       <c r="D24" s="14">
         <f>[1]Forward!D28</f>
-        <v>24.722336889160349</v>
+        <v>24.67106496040045</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A25" s="12">
         <f>[1]Forward!$C$2</f>
-        <v>46037.434039351851</v>
+        <v>46050.386261574073</v>
       </c>
       <c r="B25" s="12">
         <f>[1]Forward!B29</f>
@@ -2960,17 +2962,17 @@
       </c>
       <c r="C25" s="13">
         <f>[1]Forward!C29</f>
-        <v>27.263120769847632</v>
+        <v>27.612037432340948</v>
       </c>
       <c r="D25" s="14">
         <f>[1]Forward!D29</f>
-        <v>24.745958330253249</v>
+        <v>24.685334210569998</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A26" s="12">
         <f>[1]Forward!$C$2</f>
-        <v>46037.434039351851</v>
+        <v>46050.386261574073</v>
       </c>
       <c r="B26" s="12">
         <f>[1]Forward!B30</f>
@@ -2978,17 +2980,17 @@
       </c>
       <c r="C26" s="13">
         <f>[1]Forward!C30</f>
-        <v>27.814047145199236</v>
+        <v>28.064027084849055</v>
       </c>
       <c r="D26" s="14">
         <f>[1]Forward!D30</f>
-        <v>24.772730621634899</v>
+        <v>24.701482464614351</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A27" s="12">
         <f>[1]Forward!$C$2</f>
-        <v>46037.434039351851</v>
+        <v>46050.386261574073</v>
       </c>
       <c r="B27" s="12">
         <f>[1]Forward!B31</f>
@@ -2996,17 +2998,17 @@
       </c>
       <c r="C27" s="13">
         <f>[1]Forward!C31</f>
-        <v>27.765187711169723</v>
+        <v>28.014329469900527</v>
       </c>
       <c r="D27" s="14">
         <f>[1]Forward!D31</f>
-        <v>24.792830255214501</v>
+        <v>24.717027609701599</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A28" s="12">
         <f>[1]Forward!$C$2</f>
-        <v>46037.434039351851</v>
+        <v>46050.386261574073</v>
       </c>
       <c r="B28" s="12">
         <f>[1]Forward!B32</f>
@@ -3014,17 +3016,17 @@
       </c>
       <c r="C28" s="13">
         <f>[1]Forward!C32</f>
-        <v>27.016009722717232</v>
+        <v>27.262382948070574</v>
       </c>
       <c r="D28" s="14">
         <f>[1]Forward!D32</f>
-        <v>24.813490454096851</v>
+        <v>24.735151483676599</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A29" s="12">
         <f>[1]Forward!$C$2</f>
-        <v>46037.434039351851</v>
+        <v>46050.386261574073</v>
       </c>
       <c r="B29" s="12">
         <f>[1]Forward!B33</f>
@@ -3032,17 +3034,17 @@
       </c>
       <c r="C29" s="13">
         <f>[1]Forward!C33</f>
-        <v>25.047517413928293</v>
+        <v>24.59815863365581</v>
       </c>
       <c r="D29" s="14">
         <f>[1]Forward!D33</f>
-        <v>24.837710041818301</v>
+        <v>24.756390390477399</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A30" s="12">
         <f>[1]Forward!$C$2</f>
-        <v>46037.434039351851</v>
+        <v>46050.386261574073</v>
       </c>
       <c r="B30" s="12">
         <f>[1]Forward!B34</f>
@@ -3050,17 +3052,17 @@
       </c>
       <c r="C30" s="13">
         <f>[1]Forward!C34</f>
-        <v>24.222335861429901</v>
+        <v>23.623653227491126</v>
       </c>
       <c r="D30" s="14">
         <f>[1]Forward!D34</f>
-        <v>24.856941156696902</v>
+        <v>24.773249066614</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A31" s="12">
         <f>[1]Forward!$C$2</f>
-        <v>46037.434039351851</v>
+        <v>46050.386261574073</v>
       </c>
       <c r="B31" s="12">
         <f>[1]Forward!B35</f>
@@ -3068,17 +3070,17 @@
       </c>
       <c r="C31" s="13">
         <f>[1]Forward!C35</f>
-        <v>24.064899907334812</v>
+        <v>23.484283829048504</v>
       </c>
       <c r="D31" s="14">
         <f>[1]Forward!D35</f>
-        <v>24.879019047143849</v>
+        <v>24.792597120893653</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A32" s="12">
         <f>[1]Forward!$C$2</f>
-        <v>46037.434039351851</v>
+        <v>46050.386261574073</v>
       </c>
       <c r="B32" s="12">
         <f>[1]Forward!B36</f>
@@ -3086,17 +3088,17 @@
       </c>
       <c r="C32" s="13">
         <f>[1]Forward!C36</f>
-        <v>23.961752213272511</v>
+        <v>23.338432133003902</v>
       </c>
       <c r="D32" s="14">
         <f>[1]Forward!D36</f>
-        <v>24.901806572860252</v>
+        <v>24.812560107808899</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A33" s="12">
         <f>[1]Forward!$C$2</f>
-        <v>46037.434039351851</v>
+        <v>46050.386261574073</v>
       </c>
       <c r="B33" s="12">
         <f>[1]Forward!B37</f>
@@ -3104,17 +3106,17 @@
       </c>
       <c r="C33" s="13">
         <f>[1]Forward!C37</f>
-        <v>24.157189949390549</v>
+        <v>23.532901061063374</v>
       </c>
       <c r="D33" s="14">
         <f>[1]Forward!D37</f>
-        <v>24.922455526302649</v>
+        <v>24.830643493508649</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A34" s="12">
         <f>[1]Forward!$C$2</f>
-        <v>46037.434039351851</v>
+        <v>46050.386261574073</v>
       </c>
       <c r="B34" s="12">
         <f>[1]Forward!B38</f>
@@ -3122,17 +3124,17 @@
       </c>
       <c r="C34" s="13">
         <f>[1]Forward!C38</f>
-        <v>24.488348335590562</v>
+        <v>23.86241785583081</v>
       </c>
       <c r="D34" s="14">
         <f>[1]Forward!D38</f>
-        <v>24.944526188443298</v>
+        <v>24.849965522870448</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A35" s="12">
         <f>[1]Forward!$C$2</f>
-        <v>46037.434039351851</v>
+        <v>46050.386261574073</v>
       </c>
       <c r="B35" s="12">
         <f>[1]Forward!B39</f>
@@ -3140,17 +3142,17 @@
       </c>
       <c r="C35" s="13">
         <f>[1]Forward!C39</f>
-        <v>24.663156532896146</v>
+        <v>24.025555678814033</v>
       </c>
       <c r="D35" s="14">
         <f>[1]Forward!D39</f>
-        <v>24.966594414959097</v>
+        <v>24.869278782966401</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A36" s="12">
         <f>[1]Forward!$C$2</f>
-        <v>46037.434039351851</v>
+        <v>46050.386261574073</v>
       </c>
       <c r="B36" s="12">
         <f>[1]Forward!B40</f>
@@ -3158,17 +3160,17 @@
       </c>
       <c r="C36" s="13">
         <f>[1]Forward!C40</f>
-        <v>25.526339867417498</v>
+        <v>24.884460111076702</v>
       </c>
       <c r="D36" s="14">
         <f>[1]Forward!D40</f>
-        <v>24.98794844416085</v>
+        <v>24.887960685163051</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A37" s="12">
         <f>[1]Forward!$C$2</f>
-        <v>46037.434039351851</v>
+        <v>46050.386261574073</v>
       </c>
       <c r="B37" s="12">
         <f>[1]Forward!B41</f>
@@ -3176,17 +3178,17 @@
       </c>
       <c r="C37" s="13">
         <f>[1]Forward!C41</f>
-        <v>25.917215339653577</v>
+        <v>25.273397967195642</v>
       </c>
       <c r="D37" s="14">
         <f>[1]Forward!D41</f>
-        <v>25.009300192340248</v>
+        <v>24.906634374727851</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A38" s="12">
         <f>[1]Forward!$C$2</f>
-        <v>46037.434039351851</v>
+        <v>46050.386261574073</v>
       </c>
       <c r="B38" s="12">
         <f>[1]Forward!B42</f>
@@ -3194,17 +3196,17 @@
       </c>
       <c r="C38" s="13">
         <f>[1]Forward!C42</f>
-        <v>26.546114462368614</v>
+        <v>25.616164054954741</v>
       </c>
       <c r="D38" s="14">
         <f>[1]Forward!D42</f>
-        <v>25.0320728762049</v>
+        <v>24.926543924784902</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A39" s="12">
         <f>[1]Forward!$C$2</f>
-        <v>46037.434039351851</v>
+        <v>46050.386261574073</v>
       </c>
       <c r="B39" s="12">
         <f>[1]Forward!B43</f>
@@ -3212,17 +3214,17 @@
       </c>
       <c r="C39" s="13">
         <f>[1]Forward!C43</f>
-        <v>26.689327097970885</v>
+        <v>25.756113452002396</v>
       </c>
       <c r="D39" s="14">
         <f>[1]Forward!D43</f>
-        <v>25.053990216973801</v>
+        <v>24.945034379127549</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A40" s="12">
         <f>[1]Forward!$C$2</f>
-        <v>46037.434039351851</v>
+        <v>46050.386261574073</v>
       </c>
       <c r="B40" s="12">
         <f>[1]Forward!B44</f>
@@ -3230,17 +3232,17 @@
       </c>
       <c r="C40" s="13">
         <f>[1]Forward!C44</f>
-        <v>26.232148299702096</v>
+        <v>25.329755986578153</v>
       </c>
       <c r="D40" s="14">
         <f>[1]Forward!D44</f>
-        <v>25.074578182154902</v>
+        <v>24.9621287284691</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A41" s="12">
         <f>[1]Forward!$C$2</f>
-        <v>46037.434039351851</v>
+        <v>46050.386261574073</v>
       </c>
       <c r="B41" s="12">
         <f>[1]Forward!B45</f>
@@ -3248,17 +3250,17 @@
       </c>
       <c r="C41" s="13">
         <f>[1]Forward!C45</f>
-        <v>24.330725153167329</v>
+        <v>23.48546160688041</v>
       </c>
       <c r="D41" s="14">
         <f>[1]Forward!D45</f>
-        <v>25.098105863410151</v>
+        <v>24.981655059711898</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A42" s="12">
         <f>[1]Forward!$C$2</f>
-        <v>46037.434039351851</v>
+        <v>46050.386261574073</v>
       </c>
       <c r="B42" s="12">
         <f>[1]Forward!B46</f>
@@ -3266,17 +3268,17 @@
       </c>
       <c r="C42" s="13">
         <f>[1]Forward!C46</f>
-        <v>23.709402641785168</v>
+        <v>22.872504945392631</v>
       </c>
       <c r="D42" s="14">
         <f>[1]Forward!D46</f>
-        <v>25.119426514558249</v>
+        <v>24.999341521202751</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A43" s="12">
         <f>[1]Forward!$C$2</f>
-        <v>46037.434039351851</v>
+        <v>46050.386261574073</v>
       </c>
       <c r="B43" s="12">
         <f>[1]Forward!B47</f>
@@ -3284,17 +3286,17 @@
       </c>
       <c r="C43" s="13">
         <f>[1]Forward!C47</f>
-        <v>23.092486673036927</v>
+        <v>22.270397074373665</v>
       </c>
       <c r="D43" s="14">
         <f>[1]Forward!D47</f>
-        <v>25.14221617806335</v>
+        <v>25.018237985278951</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A44" s="12">
         <f>[1]Forward!$C$2</f>
-        <v>46037.434039351851</v>
+        <v>46050.386261574073</v>
       </c>
       <c r="B44" s="12">
         <f>[1]Forward!B48</f>
@@ -3302,17 +3304,17 @@
       </c>
       <c r="C44" s="13">
         <f>[1]Forward!C48</f>
-        <v>22.971306750604239</v>
+        <v>22.156484774451155</v>
       </c>
       <c r="D44" s="14">
         <f>[1]Forward!D48</f>
-        <v>25.165004418278698</v>
+        <v>25.037124370863001</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A45" s="12">
         <f>[1]Forward!$C$2</f>
-        <v>46037.434039351851</v>
+        <v>46050.386261574073</v>
       </c>
       <c r="B45" s="12">
         <f>[1]Forward!B49</f>
@@ -3320,17 +3322,17 @@
       </c>
       <c r="C45" s="13">
         <f>[1]Forward!C49</f>
-        <v>23.197142060592434</v>
+        <v>22.422280140937008</v>
       </c>
       <c r="D45" s="14">
         <f>[1]Forward!D49</f>
-        <v>25.187056198809351</v>
+        <v>25.055391922135549</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A46" s="12">
         <f>[1]Forward!$C$2</f>
-        <v>46037.434039351851</v>
+        <v>46050.386261574073</v>
       </c>
       <c r="B46" s="12">
         <f>[1]Forward!B50</f>
@@ -3338,17 +3340,17 @@
       </c>
       <c r="C46" s="13">
         <f>[1]Forward!C50</f>
-        <v>23.654320858861222</v>
+        <v>22.943022083439899</v>
       </c>
       <c r="D46" s="14">
         <f>[1]Forward!D50</f>
-        <v>25.211311617840749</v>
+        <v>25.075475326774001</v>
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A47" s="12">
         <f>[1]Forward!$C$2</f>
-        <v>46037.434039351851</v>
+        <v>46050.386261574073</v>
       </c>
       <c r="B47" s="12">
         <f>[1]Forward!B51</f>
@@ -3356,17 +3358,17 @@
       </c>
       <c r="C47" s="13">
         <f>[1]Forward!C51</f>
-        <v>24.115906199763923</v>
+        <v>23.340087814598355</v>
       </c>
       <c r="D47" s="14">
         <f>[1]Forward!D51</f>
-        <v>25.23189070856505</v>
+        <v>25.092506834986651</v>
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A48" s="12">
         <f>[1]Forward!$C$2</f>
-        <v>46037.434039351851</v>
+        <v>46050.386261574073</v>
       </c>
       <c r="B48" s="12">
         <f>[1]Forward!B52</f>
@@ -3374,17 +3376,17 @@
       </c>
       <c r="C48" s="13">
         <f>[1]Forward!C52</f>
-        <v>24.540035928278343</v>
+        <v>23.817434595226008</v>
       </c>
       <c r="D48" s="14">
         <f>[1]Forward!D52</f>
-        <v>25.254673347446051</v>
+        <v>25.111353556827549</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A49" s="12">
         <f>[1]Forward!$C$2</f>
-        <v>46037.434039351851</v>
+        <v>46050.386261574073</v>
       </c>
       <c r="B49" s="12">
         <f>[1]Forward!B53</f>
@@ -3392,11 +3394,11 @@
       </c>
       <c r="C49" s="13">
         <f>[1]Forward!C53</f>
-        <v>24.909083873868809</v>
+        <v>24.186293471165552</v>
       </c>
       <c r="D49" s="14">
         <f>[1]Forward!D53</f>
-        <v>25.278189417262599</v>
+        <v>25.1307976660325</v>
       </c>
     </row>
   </sheetData>

</xml_diff>